<commit_message>
reordering and comment cleanup
</commit_message>
<xml_diff>
--- a/src/generated_files/MP4_iTunes_ffmpeg_mapping.xlsx
+++ b/src/generated_files/MP4_iTunes_ffmpeg_mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MusicProcessing\src\generated_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05B2C3FB-B136-4525-8253-FEC572C941AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40C0D274-1D22-4FB7-8FE1-97E175E46C5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="134">
   <si>
     <t>iTunes Element</t>
   </si>
@@ -210,9 +210,6 @@
     <t>trkn</t>
   </si>
   <si>
-    <t>binary</t>
-  </si>
-  <si>
     <t>Disc Number</t>
   </si>
   <si>
@@ -400,6 +397,36 @@
   </si>
   <si>
     <t>Notes</t>
+  </si>
+  <si>
+    <t>tuple of 2 ints</t>
+  </si>
+  <si>
+    <t>-metadata track=""</t>
+  </si>
+  <si>
+    <t>-metadata disc=""</t>
+  </si>
+  <si>
+    <t>-metadata tempo=""</t>
+  </si>
+  <si>
+    <t>-metadata sort=""</t>
+  </si>
+  <si>
+    <t>-metadata cover=""</t>
+  </si>
+  <si>
+    <t>-metadata encoded=""</t>
+  </si>
+  <si>
+    <t>-metadata content=""</t>
+  </si>
+  <si>
+    <t>track</t>
+  </si>
+  <si>
+    <t>disc</t>
   </si>
 </sst>
 </file>
@@ -876,7 +903,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
@@ -896,7 +923,7 @@
         <v>10</v>
       </c>
       <c r="G2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -916,7 +943,7 @@
         <v>14</v>
       </c>
       <c r="G3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -1001,7 +1028,7 @@
         <v>8</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>34</v>
@@ -1021,7 +1048,7 @@
         <v>8</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>38</v>
@@ -1041,7 +1068,7 @@
         <v>8</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>42</v>
@@ -1061,7 +1088,7 @@
         <v>8</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>46</v>
@@ -1089,7 +1116,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B13" t="s">
         <v>52</v>
@@ -1098,7 +1125,7 @@
         <v>8</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E13" t="s">
         <v>51</v>
@@ -1135,243 +1162,282 @@
         <v>60</v>
       </c>
       <c r="C15" t="s">
-        <v>61</v>
+        <v>124</v>
+      </c>
+      <c r="E15" t="s">
+        <v>132</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
+        <v>61</v>
+      </c>
+      <c r="B16" t="s">
         <v>62</v>
       </c>
-      <c r="B16" t="s">
-        <v>63</v>
-      </c>
       <c r="C16" t="s">
-        <v>61</v>
+        <v>124</v>
+      </c>
+      <c r="E16" t="s">
+        <v>133</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
+        <v>63</v>
+      </c>
+      <c r="B17" t="s">
         <v>64</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>65</v>
       </c>
-      <c r="C17" t="s">
-        <v>66</v>
+      <c r="F17" s="1" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
+        <v>66</v>
+      </c>
+      <c r="B18" t="s">
         <v>67</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
         <v>68</v>
       </c>
-      <c r="C18" t="s">
+      <c r="E18" t="s">
         <v>69</v>
       </c>
-      <c r="E18" t="s">
+      <c r="F18" s="1" t="s">
         <v>70</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
+        <v>71</v>
+      </c>
+      <c r="B19" t="s">
         <v>72</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" t="s">
+        <v>8</v>
+      </c>
+      <c r="D19" t="s">
+        <v>122</v>
+      </c>
+      <c r="E19" t="s">
         <v>73</v>
       </c>
-      <c r="C19" t="s">
-        <v>8</v>
-      </c>
-      <c r="D19" t="s">
-        <v>123</v>
-      </c>
-      <c r="E19" t="s">
+      <c r="F19" s="1" t="s">
         <v>74</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
+        <v>75</v>
+      </c>
+      <c r="B20" t="s">
         <v>76</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
+        <v>8</v>
+      </c>
+      <c r="D20" t="s">
         <v>77</v>
       </c>
-      <c r="C20" t="s">
-        <v>8</v>
-      </c>
-      <c r="D20" t="s">
+      <c r="E20" t="s">
         <v>78</v>
       </c>
-      <c r="E20" t="s">
+      <c r="F20" s="1" t="s">
         <v>79</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
+        <v>80</v>
+      </c>
+      <c r="B21" t="s">
         <v>81</v>
       </c>
-      <c r="B21" t="s">
-        <v>82</v>
-      </c>
       <c r="C21" t="s">
         <v>8</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
+        <v>82</v>
+      </c>
+      <c r="B22" t="s">
         <v>83</v>
       </c>
-      <c r="B22" t="s">
-        <v>84</v>
-      </c>
       <c r="C22" t="s">
         <v>8</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
+        <v>84</v>
+      </c>
+      <c r="B23" t="s">
         <v>85</v>
       </c>
-      <c r="B23" t="s">
-        <v>86</v>
-      </c>
       <c r="C23" t="s">
         <v>8</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
+        <v>86</v>
+      </c>
+      <c r="B24" t="s">
         <v>87</v>
       </c>
-      <c r="B24" t="s">
-        <v>88</v>
-      </c>
       <c r="C24" t="s">
         <v>8</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
+        <v>88</v>
+      </c>
+      <c r="B25" t="s">
         <v>89</v>
       </c>
-      <c r="B25" t="s">
-        <v>90</v>
-      </c>
       <c r="C25" t="s">
         <v>8</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
+        <v>90</v>
+      </c>
+      <c r="B26" t="s">
         <v>91</v>
       </c>
-      <c r="B26" t="s">
+      <c r="C26" t="s">
         <v>92</v>
       </c>
-      <c r="C26" t="s">
+      <c r="D26" t="s">
         <v>93</v>
       </c>
-      <c r="D26" t="s">
-        <v>94</v>
+      <c r="F26" s="1" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
+        <v>94</v>
+      </c>
+      <c r="B27" t="s">
         <v>95</v>
       </c>
-      <c r="B27" t="s">
+      <c r="C27" t="s">
+        <v>8</v>
+      </c>
+      <c r="D27" t="s">
         <v>96</v>
       </c>
-      <c r="C27" t="s">
-        <v>8</v>
-      </c>
-      <c r="D27" t="s">
+      <c r="E27" t="s">
         <v>97</v>
       </c>
-      <c r="E27" t="s">
+      <c r="F27" s="1" t="s">
         <v>98</v>
-      </c>
-      <c r="F27" s="1" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
+        <v>99</v>
+      </c>
+      <c r="B28" t="s">
         <v>100</v>
       </c>
-      <c r="B28" t="s">
+      <c r="C28" t="s">
+        <v>8</v>
+      </c>
+      <c r="D28" t="s">
         <v>101</v>
       </c>
-      <c r="C28" t="s">
-        <v>8</v>
-      </c>
-      <c r="D28" t="s">
+      <c r="E28" t="s">
         <v>102</v>
       </c>
-      <c r="E28" t="s">
+      <c r="F28" s="1" t="s">
         <v>103</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
+        <v>104</v>
+      </c>
+      <c r="B29" t="s">
         <v>105</v>
       </c>
-      <c r="B29" t="s">
+      <c r="C29" t="s">
+        <v>8</v>
+      </c>
+      <c r="D29" t="s">
         <v>106</v>
       </c>
-      <c r="C29" t="s">
-        <v>8</v>
-      </c>
-      <c r="D29" t="s">
-        <v>107</v>
+      <c r="F29" s="1" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
+        <v>107</v>
+      </c>
+      <c r="B30" t="s">
         <v>108</v>
       </c>
-      <c r="B30" t="s">
+      <c r="C30" t="s">
         <v>109</v>
       </c>
-      <c r="C30" t="s">
+      <c r="D30" t="s">
         <v>110</v>
       </c>
-      <c r="D30" t="s">
+      <c r="E30" t="s">
         <v>111</v>
       </c>
-      <c r="E30" t="s">
+      <c r="F30" s="1" t="s">
         <v>112</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
+        <v>113</v>
+      </c>
+      <c r="B31" t="s">
         <v>114</v>
       </c>
-      <c r="B31" t="s">
+      <c r="C31" t="s">
         <v>115</v>
       </c>
-      <c r="C31" t="s">
+      <c r="D31" t="s">
         <v>116</v>
       </c>
-      <c r="D31" t="s">
-        <v>117</v>
+      <c r="F31" s="1" t="s">
+        <v>131</v>
       </c>
     </row>
   </sheetData>

</xml_diff>